<commit_message>
Group OLX fallback images by listing
</commit_message>
<xml_diff>
--- a/Dataset/rooms_dataset.xlsx
+++ b/Dataset/rooms_dataset.xlsx
@@ -422,15 +422,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M231"/>
+  <dimension ref="A1:M149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -7635,10 +7635,26 @@
           <t>room_120_img1.webp</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>room_120_img2.webp</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>room_120_img3.webp</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>room_120_img4.webp</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>room_120_img5.webp</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr">
         <is>
           <t>Mannu Chowk, Bilaspur</t>
@@ -7682,10 +7698,26 @@
           <t>room_121_img1.webp</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>room_121_img2.webp</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>room_121_img3.webp</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>room_121_img4.webp</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>room_121_img5.webp</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr">
         <is>
           <t>Raj Kishore Nagar, Bilaspur</t>
@@ -7780,8 +7812,16 @@
           <t>room_123_img1.webp</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>room_123_img2.webp</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>room_123_img3.webp</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -7827,10 +7867,26 @@
           <t>room_124_img1.webp</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>room_124_img2.webp</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>room_124_img3.webp</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>room_124_img4.webp</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>room_124_img5.webp</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr">
         <is>
           <t>Sarkanda, Bilaspur</t>
@@ -7874,8 +7930,16 @@
           <t>room_125_img1.webp</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>room_125_img2.webp</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>room_125_img3.webp</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -7921,10 +7985,26 @@
           <t>room_126_img1.webp</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>room_126_img2.webp</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>room_126_img3.webp</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>room_126_img4.webp</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>room_126_img5.webp</t>
+        </is>
+      </c>
       <c r="G127" t="inlineStr">
         <is>
           <t>Balram Talkies Chowk, Bilaspur</t>
@@ -7968,8 +8048,16 @@
           <t>room_127_img1.webp</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
-      <c r="D128" t="inlineStr"/>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>room_127_img2.webp</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>room_127_img3.webp</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -8015,10 +8103,26 @@
           <t>room_128_img1.webp</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
-      <c r="D129" t="inlineStr"/>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>room_128_img2.webp</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>room_128_img3.webp</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>room_128_img4.webp</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>room_128_img5.webp</t>
+        </is>
+      </c>
       <c r="G129" t="inlineStr">
         <is>
           <t>Abhishek Vihar, Bilaspur</t>
@@ -8062,8 +8166,16 @@
           <t>room_129_img1.webp</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
-      <c r="D130" t="inlineStr"/>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>room_129_img2.webp</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>room_129_img3.webp</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -8109,10 +8221,26 @@
           <t>room_130_img1.webp</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
-      <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>room_130_img2.webp</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>room_130_img3.webp</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>room_130_img4.webp</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>room_130_img5.webp</t>
+        </is>
+      </c>
       <c r="G131" t="inlineStr">
         <is>
           <t>Sarkanda, Bilaspur</t>
@@ -8156,10 +8284,26 @@
           <t>room_131_img1.webp</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
-      <c r="D132" t="inlineStr"/>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>room_131_img2.webp</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>room_131_img3.webp</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>room_131_img4.webp</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>room_131_img5.webp</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr">
         <is>
           <t>Vivekanand Nagar, Bilaspur</t>
@@ -8203,10 +8347,26 @@
           <t>room_132_img1.webp</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
-      <c r="D133" t="inlineStr"/>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>room_132_img2.webp</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>room_132_img3.webp</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>room_132_img4.webp</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>room_132_img5.webp</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
           <t>Babji Nagar, Bilaspur</t>
@@ -8250,10 +8410,26 @@
           <t>room_133_img1.webp</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
-      <c r="D134" t="inlineStr"/>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>room_133_img2.webp</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>room_133_img3.webp</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>room_133_img4.webp</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>room_133_img5.webp</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
           <t>Bandhwapara, Bilaspur</t>
@@ -8297,10 +8473,26 @@
           <t>room_134_img1.webp</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>room_134_img2.webp</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>room_134_img3.webp</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>room_134_img4.webp</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>room_134_img5.webp</t>
+        </is>
+      </c>
       <c r="G135" t="inlineStr">
         <is>
           <t>Raj Kishore Nagar, Bilaspur</t>
@@ -8344,8 +8536,16 @@
           <t>room_135_img1.webp</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>room_135_img2.webp</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>room_135_img3.webp</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -8391,9 +8591,21 @@
           <t>room_136_img1.webp</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>room_136_img2.webp</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>room_136_img3.webp</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>room_136_img4.webp</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
@@ -8442,9 +8654,21 @@
           <t>room_137_img1.webp</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr"/>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>room_137_img2.webp</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>room_137_img3.webp</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>room_137_img4.webp</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
@@ -8489,10 +8713,26 @@
           <t>room_138_img1.webp</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>room_138_img2.webp</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>room_138_img3.webp</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>room_138_img4.webp</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>room_138_img5.webp</t>
+        </is>
+      </c>
       <c r="G139" t="inlineStr">
         <is>
           <t>Dayalband, Bilaspur</t>
@@ -8536,7 +8776,11 @@
           <t>room_139_img1.webp</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>room_139_img2.webp</t>
+        </is>
+      </c>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr"/>
@@ -8583,10 +8827,26 @@
           <t>room_140_img1.webp</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>room_140_img2.webp</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>room_140_img3.webp</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>room_140_img4.webp</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>room_140_img5.webp</t>
+        </is>
+      </c>
       <c r="G141" t="inlineStr">
         <is>
           <t>Mangla, Bilaspur</t>
@@ -8630,10 +8890,26 @@
           <t>room_141_img1.webp</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>room_141_img2.webp</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>room_141_img3.webp</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>room_141_img4.webp</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>room_141_img5.webp</t>
+        </is>
+      </c>
       <c r="G142" t="inlineStr">
         <is>
           <t>Mannu Chowk, Bilaspur</t>
@@ -8677,10 +8953,26 @@
           <t>room_142_img1.webp</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>room_142_img2.webp</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>room_142_img3.webp</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>room_142_img4.webp</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>room_142_img5.webp</t>
+        </is>
+      </c>
       <c r="G143" t="inlineStr">
         <is>
           <t>Raj Kishore Nagar, Bilaspur</t>
@@ -8724,10 +9016,26 @@
           <t>room_143_img1.webp</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>room_143_img2.webp</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>room_143_img3.webp</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>room_143_img4.webp</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>room_143_img5.webp</t>
+        </is>
+      </c>
       <c r="G144" t="inlineStr">
         <is>
           <t>Sarkanda, Bilaspur</t>
@@ -8869,10 +9177,26 @@
           <t>room_146_img1.webp</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>room_146_img2.webp</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>room_146_img3.webp</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>room_146_img4.webp</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>room_146_img5.webp</t>
+        </is>
+      </c>
       <c r="G147" t="inlineStr">
         <is>
           <t>Hamu Nagar, Bilaspur</t>
@@ -8963,7 +9287,11 @@
           <t>room_148_img1.webp</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>room_148_img2.webp</t>
+        </is>
+      </c>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
@@ -8999,3880 +9327,6 @@
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>149</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>room_149_img1.webp</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>Sarkanda, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M150" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>room_150_img1.webp</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr"/>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>27 Kholi, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>151</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>room_151_img1.webp</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>Agyeya Nagar, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M152" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>room_152_img1.webp</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>Juna Bilaspur, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr"/>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>4600</t>
-        </is>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>153</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>room_153_img1.webp</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>Sarkanda, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>154</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>room_154_img1.webp</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
-      <c r="E155" t="inlineStr"/>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>Jarhabhata, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>440</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="M155" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>155</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>room_155_img1.webp</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr"/>
-      <c r="D156" t="inlineStr"/>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>Tiphara, Tifra</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="M156" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>room_156_img1.webp</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr"/>
-      <c r="D157" t="inlineStr"/>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>Bengali Para, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr"/>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>6500</t>
-        </is>
-      </c>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>room_157_img1.webp</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr"/>
-      <c r="D158" t="inlineStr"/>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Nehru Nagar, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J158" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K158" t="inlineStr"/>
-      <c r="L158" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M158" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>room_158_img1.webp</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Godpara, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K159" t="inlineStr"/>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M159" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>159</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>room_159_img1.webp</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr"/>
-      <c r="D160" t="inlineStr"/>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>Gandhi Chowk, Bilaspur</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr">
-        <is>
-          <t>4500</t>
-        </is>
-      </c>
-      <c r="M160" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>room_160_img1.webp</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr"/>
-      <c r="D161" t="inlineStr"/>
-      <c r="E161" t="inlineStr"/>
-      <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>Telibandha, Raipur</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="I161" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>4500</t>
-        </is>
-      </c>
-      <c r="M161" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>161</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>room_161_img1.webp</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr"/>
-      <c r="D162" t="inlineStr"/>
-      <c r="E162" t="inlineStr"/>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>Mowa, Raipur</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M162" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>162</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>room_162_img1.webp</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr"/>
-      <c r="D163" t="inlineStr"/>
-      <c r="E163" t="inlineStr"/>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>Nahar Para, Raipur</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J163" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr">
-        <is>
-          <t>2700</t>
-        </is>
-      </c>
-      <c r="M163" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>room_163_img1.webp</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr"/>
-      <c r="D164" t="inlineStr"/>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>Pandri, Raipur</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J164" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr">
-        <is>
-          <t>3250</t>
-        </is>
-      </c>
-      <c r="M164" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>164</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>room_164_img1.webp</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>Rajiv Nagar Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="I165" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J165" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M165" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>room_165_img1.webp</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr"/>
-      <c r="D166" t="inlineStr"/>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>Kabeer Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J166" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M166" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>166</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>room_166_img1.webp</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr"/>
-      <c r="D167" t="inlineStr"/>
-      <c r="E167" t="inlineStr"/>
-      <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>Pachpedi Naka, Raipur</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>furnished</t>
-        </is>
-      </c>
-      <c r="J167" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr">
-        <is>
-          <t>4300</t>
-        </is>
-      </c>
-      <c r="M167" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>room_167_img1.webp</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr"/>
-      <c r="D168" t="inlineStr"/>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>Kota, Raipur</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J168" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M168" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>168</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>room_168_img1.webp</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr"/>
-      <c r="D169" t="inlineStr"/>
-      <c r="E169" t="inlineStr"/>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>Pachpedi Naka, Raipur</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J169" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M169" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>room_169_img1.webp</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr"/>
-      <c r="D170" t="inlineStr"/>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>Shyam Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J170" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr">
-        <is>
-          <t>6500</t>
-        </is>
-      </c>
-      <c r="M170" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>room_170_img1.webp</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr"/>
-      <c r="D171" t="inlineStr"/>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>Shyam Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>7000</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>furnished</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="L171" t="inlineStr">
-        <is>
-          <t>150000</t>
-        </is>
-      </c>
-      <c r="M171" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>171</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>room_171_img1.webp</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr"/>
-      <c r="D172" t="inlineStr"/>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>Danganiya, Raipur</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr">
-        <is>
-          <t>2600</t>
-        </is>
-      </c>
-      <c r="M172" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>172</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>room_172_img1.webp</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr"/>
-      <c r="D173" t="inlineStr"/>
-      <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>Kotwali Chowk, Raipur</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="M173" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>173</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>room_173_img1.webp</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr"/>
-      <c r="D174" t="inlineStr"/>
-      <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>Matpara, Raipur</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>650</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M174" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>174</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>room_174_img1.webp</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr"/>
-      <c r="D175" t="inlineStr"/>
-      <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>Deendayal Upadhyaya Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M175" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>175</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>room_175_img1.webp</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr"/>
-      <c r="D176" t="inlineStr"/>
-      <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>Avanti Vihar Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M176" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>room_176_img1.webp</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr"/>
-      <c r="D177" t="inlineStr"/>
-      <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>Mowa, Raipur</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr">
-        <is>
-          <t>7000</t>
-        </is>
-      </c>
-      <c r="M177" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>177</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>room_177_img1.webp</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>Kota, Raipur</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr">
-        <is>
-          <t>4700</t>
-        </is>
-      </c>
-      <c r="M178" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>178</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>room_178_img1.webp</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr"/>
-      <c r="D179" t="inlineStr"/>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>Kanchanjanga Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J179" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K179" t="inlineStr"/>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M179" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>179</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>room_179_img1.webp</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr"/>
-      <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>Mowa, Raipur</t>
-        </is>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J180" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr">
-        <is>
-          <t>3100</t>
-        </is>
-      </c>
-      <c r="M180" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>room_180_img1.webp</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr"/>
-      <c r="D181" t="inlineStr"/>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>Pandri, Raipur</t>
-        </is>
-      </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J181" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K181" t="inlineStr"/>
-      <c r="L181" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="M181" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>181</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>room_181_img1.webp</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr"/>
-      <c r="D182" t="inlineStr"/>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>Pandri, Raipur</t>
-        </is>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J182" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K182" t="inlineStr"/>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t>3250</t>
-        </is>
-      </c>
-      <c r="M182" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>182</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>room_182_img1.webp</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr"/>
-      <c r="D183" t="inlineStr"/>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>Pachpedi Naka, Raipur</t>
-        </is>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>650</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J183" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K183" t="inlineStr"/>
-      <c r="L183" t="inlineStr">
-        <is>
-          <t>5500</t>
-        </is>
-      </c>
-      <c r="M183" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>183</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>room_183_img1.webp</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr"/>
-      <c r="D184" t="inlineStr"/>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>Mangal Bazar, Raipur</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>280</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J184" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M184" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>184</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>room_184_img1.webp</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr"/>
-      <c r="D185" t="inlineStr"/>
-      <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>Kota, Raipur</t>
-        </is>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J185" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="inlineStr">
-        <is>
-          <t>7000</t>
-        </is>
-      </c>
-      <c r="M185" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>185</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>room_185_img1.webp</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr"/>
-      <c r="D186" t="inlineStr"/>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>Mangal Bazar, Raipur</t>
-        </is>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J186" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="inlineStr">
-        <is>
-          <t>2900</t>
-        </is>
-      </c>
-      <c r="M186" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>186</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>room_186_img1.webp</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr"/>
-      <c r="D187" t="inlineStr"/>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>Mahavir Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>850</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J187" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="inlineStr">
-        <is>
-          <t>13000</t>
-        </is>
-      </c>
-      <c r="M187" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>187</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>room_187_img1.webp</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr"/>
-      <c r="D188" t="inlineStr"/>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>Ravi Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J188" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="M188" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>188</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>room_188_img1.webp</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr"/>
-      <c r="D189" t="inlineStr"/>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>Fafadih, Raipur</t>
-        </is>
-      </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>furnished</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K189" t="inlineStr"/>
-      <c r="L189" t="inlineStr">
-        <is>
-          <t>5500</t>
-        </is>
-      </c>
-      <c r="M189" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>189</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>room_189_img1.webp</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr"/>
-      <c r="D190" t="inlineStr"/>
-      <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr"/>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>Sunder Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I190" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K190" t="inlineStr"/>
-      <c r="L190" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M190" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>190</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>room_190_img1.webp</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr"/>
-      <c r="D191" t="inlineStr"/>
-      <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr"/>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>Professor Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>3750</t>
-        </is>
-      </c>
-      <c r="I191" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K191" t="inlineStr"/>
-      <c r="L191" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M191" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>191</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>room_191_img1.webp</t>
-        </is>
-      </c>
-      <c r="C192" t="inlineStr"/>
-      <c r="D192" t="inlineStr"/>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>New Shanti Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>4500</t>
-        </is>
-      </c>
-      <c r="M192" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>192</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>room_192_img1.webp</t>
-        </is>
-      </c>
-      <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>Bhanpuri, Raipur</t>
-        </is>
-      </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="I193" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr">
-        <is>
-          <t>3800</t>
-        </is>
-      </c>
-      <c r="M193" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>193</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>room_193_img1.webp</t>
-        </is>
-      </c>
-      <c r="C194" t="inlineStr"/>
-      <c r="D194" t="inlineStr"/>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr">
-        <is>
-          <t>Gopiapara, Raipur</t>
-        </is>
-      </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I194" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K194" t="inlineStr"/>
-      <c r="L194" t="inlineStr">
-        <is>
-          <t>2800</t>
-        </is>
-      </c>
-      <c r="M194" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>194</t>
-        </is>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>room_194_img1.webp</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr"/>
-      <c r="D195" t="inlineStr"/>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>Pandri, Raipur</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K195" t="inlineStr"/>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t>3250</t>
-        </is>
-      </c>
-      <c r="M195" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>195</t>
-        </is>
-      </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>room_195_img1.webp</t>
-        </is>
-      </c>
-      <c r="C196" t="inlineStr"/>
-      <c r="D196" t="inlineStr"/>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr">
-        <is>
-          <t>New Rajendra Nagar, Raipur</t>
-        </is>
-      </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="I196" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K196" t="inlineStr"/>
-      <c r="L196" t="inlineStr">
-        <is>
-          <t>7000</t>
-        </is>
-      </c>
-      <c r="M196" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>room_196_img1.webp</t>
-        </is>
-      </c>
-      <c r="C197" t="inlineStr"/>
-      <c r="D197" t="inlineStr"/>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
-      <c r="G197" t="inlineStr">
-        <is>
-          <t>Avanti Vihar Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="I197" t="inlineStr">
-        <is>
-          <t>furnished</t>
-        </is>
-      </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K197" t="inlineStr"/>
-      <c r="L197" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
-      </c>
-      <c r="M197" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>197</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>room_197_img1.webp</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr"/>
-      <c r="D198" t="inlineStr"/>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t>Kota Colony, Raipur</t>
-        </is>
-      </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I198" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K198" t="inlineStr"/>
-      <c r="L198" t="inlineStr">
-        <is>
-          <t>7500</t>
-        </is>
-      </c>
-      <c r="M198" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>198</t>
-        </is>
-      </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>room_198_img1.webp</t>
-        </is>
-      </c>
-      <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>Mominpara, Raipur</t>
-        </is>
-      </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="I199" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K199" t="inlineStr"/>
-      <c r="L199" t="inlineStr">
-        <is>
-          <t>6500</t>
-        </is>
-      </c>
-      <c r="M199" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>199</t>
-        </is>
-      </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>room_199_img1.webp</t>
-        </is>
-      </c>
-      <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr">
-        <is>
-          <t>Telibandha, Raipur</t>
-        </is>
-      </c>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I200" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K200" t="inlineStr"/>
-      <c r="L200" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="M200" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>room_200_img1.webp</t>
-        </is>
-      </c>
-      <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>Supele Market, Bhilai</t>
-        </is>
-      </c>
-      <c r="H201" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I201" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K201" t="inlineStr"/>
-      <c r="L201" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M201" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>201</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>room_201_img1.webp</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr">
-        <is>
-          <t>Kripal Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H202" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="I202" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>2800</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>202</t>
-        </is>
-      </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>room_202_img1.webp</t>
-        </is>
-      </c>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr">
-        <is>
-          <t>Jamul, Bhilai</t>
-        </is>
-      </c>
-      <c r="H203" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="I203" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J203" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M203" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>203</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>room_203_img1.webp</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr"/>
-      <c r="D204" t="inlineStr"/>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>Shanti Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M204" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>204</t>
-        </is>
-      </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>room_204_img1.webp</t>
-        </is>
-      </c>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>Ram nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H205" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I205" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J205" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M205" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>205</t>
-        </is>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>room_205_img1.webp</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr"/>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr">
-        <is>
-          <t>Vaishali Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H206" t="inlineStr">
-        <is>
-          <t>1760</t>
-        </is>
-      </c>
-      <c r="I206" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M206" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>room_206_img1.webp</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr">
-        <is>
-          <t>Kripal Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H207" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J207" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K207" t="inlineStr"/>
-      <c r="L207" t="inlineStr">
-        <is>
-          <t>4500</t>
-        </is>
-      </c>
-      <c r="M207" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>room_207_img1.webp</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr"/>
-      <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr">
-        <is>
-          <t>Housing Board Colony, Bhilai</t>
-        </is>
-      </c>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="I208" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M208" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>room_208_img1.webp</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>Ram nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H209" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J209" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>Kitchen</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>209</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>room_209_img1.webp</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr"/>
-      <c r="D210" t="inlineStr"/>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr">
-        <is>
-          <t>Vaishali Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H210" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>furnished</t>
-        </is>
-      </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K210" t="inlineStr"/>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>6000</t>
-        </is>
-      </c>
-      <c r="M210" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>210</t>
-        </is>
-      </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>room_210_img1.webp</t>
-        </is>
-      </c>
-      <c r="C211" t="inlineStr"/>
-      <c r="D211" t="inlineStr"/>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr">
-        <is>
-          <t>Kripal Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H211" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="I211" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J211" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K211" t="inlineStr"/>
-      <c r="L211" t="inlineStr">
-        <is>
-          <t>7800</t>
-        </is>
-      </c>
-      <c r="M211" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>211</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>room_211_img1.webp</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr">
-        <is>
-          <t>Supele Market, Bhilai</t>
-        </is>
-      </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="I212" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J212" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M212" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>212</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>room_212_img1.webp</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr">
-        <is>
-          <t>Kohka Colony, Bhilai</t>
-        </is>
-      </c>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I213" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K213" t="inlineStr"/>
-      <c r="L213" t="inlineStr">
-        <is>
-          <t>5500</t>
-        </is>
-      </c>
-      <c r="M213" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>213</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>room_213_img1.webp</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr">
-        <is>
-          <t>Radhika Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K214" t="inlineStr">
-        <is>
-          <t>Kitchen</t>
-        </is>
-      </c>
-      <c r="L214" t="inlineStr">
-        <is>
-          <t>3800</t>
-        </is>
-      </c>
-      <c r="M214" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>214</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>room_214_img1.webp</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr">
-        <is>
-          <t>Hind Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H215" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K215" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t>8000</t>
-        </is>
-      </c>
-      <c r="M215" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>room_215_img1.webp</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr">
-        <is>
-          <t>Arya Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K216" t="inlineStr"/>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M216" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>216</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>room_216_img1.webp</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr"/>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
-      <c r="G217" t="inlineStr">
-        <is>
-          <t>Arya Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H217" t="inlineStr">
-        <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="I217" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J217" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K217" t="inlineStr"/>
-      <c r="L217" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M217" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>217</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>room_217_img1.webp</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr"/>
-      <c r="D218" t="inlineStr"/>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
-      <c r="G218" t="inlineStr">
-        <is>
-          <t>Nehru Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I218" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J218" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K218" t="inlineStr"/>
-      <c r="L218" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M218" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>218</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>room_218_img1.webp</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr"/>
-      <c r="D219" t="inlineStr"/>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>Kurud, Bhilai</t>
-        </is>
-      </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="I219" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J219" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K219" t="inlineStr"/>
-      <c r="L219" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M219" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>219</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>room_219_img1.webp</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr"/>
-      <c r="D220" t="inlineStr"/>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr">
-        <is>
-          <t>Maitri nagar Near Dixit Colony, Bhilai</t>
-        </is>
-      </c>
-      <c r="H220" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="I220" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J220" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr">
-        <is>
-          <t>4000</t>
-        </is>
-      </c>
-      <c r="M220" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>220</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>room_220_img1.webp</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr"/>
-      <c r="D221" t="inlineStr"/>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
-      <c r="G221" t="inlineStr">
-        <is>
-          <t>Shanti Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I221" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J221" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr">
-        <is>
-          <t>4500</t>
-        </is>
-      </c>
-      <c r="M221" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>221</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>room_221_img1.webp</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr"/>
-      <c r="D222" t="inlineStr"/>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>Panchsheel Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
-      </c>
-      <c r="I222" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J222" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M222" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>222</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>room_222_img1.webp</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr"/>
-      <c r="D223" t="inlineStr"/>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>Junwani, Bhilai</t>
-        </is>
-      </c>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>3200</t>
-        </is>
-      </c>
-      <c r="I223" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J223" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr">
-        <is>
-          <t>2100</t>
-        </is>
-      </c>
-      <c r="M223" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>223</t>
-        </is>
-      </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>room_223_img1.webp</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr"/>
-      <c r="D224" t="inlineStr"/>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>Smriti Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H224" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="I224" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J224" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K224" t="inlineStr"/>
-      <c r="L224" t="inlineStr">
-        <is>
-          <t>3000</t>
-        </is>
-      </c>
-      <c r="M224" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>224</t>
-        </is>
-      </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>room_224_img1.webp</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr"/>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr">
-        <is>
-          <t>Smriti Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="I225" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J225" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K225" t="inlineStr"/>
-      <c r="L225" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="M225" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>225</t>
-        </is>
-      </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>room_225_img1.webp</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr"/>
-      <c r="D226" t="inlineStr"/>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
-      <c r="G226" t="inlineStr">
-        <is>
-          <t>Awadhpuri Risali, Bhilai</t>
-        </is>
-      </c>
-      <c r="H226" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I226" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J226" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K226" t="inlineStr"/>
-      <c r="L226" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M226" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>room_226_img1.webp</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>Pushpak Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I227" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J227" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K227" t="inlineStr"/>
-      <c r="L227" t="inlineStr">
-        <is>
-          <t>5500</t>
-        </is>
-      </c>
-      <c r="M227" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>227</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>room_227_img1.webp</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>Madhuban Nagar, Durg</t>
-        </is>
-      </c>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="I228" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J228" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K228" t="inlineStr">
-        <is>
-          <t>Kitchen</t>
-        </is>
-      </c>
-      <c r="L228" t="inlineStr">
-        <is>
-          <t>10500</t>
-        </is>
-      </c>
-      <c r="M228" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>228</t>
-        </is>
-      </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>room_228_img1.webp</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr">
-        <is>
-          <t>Nehru Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H229" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I229" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J229" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K229" t="inlineStr"/>
-      <c r="L229" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="M229" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>229</t>
-        </is>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>room_229_img1.webp</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr"/>
-      <c r="D230" t="inlineStr"/>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr">
-        <is>
-          <t>Maitri Kunj, Bhilai</t>
-        </is>
-      </c>
-      <c r="H230" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="I230" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J230" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K230" t="inlineStr"/>
-      <c r="L230" t="inlineStr">
-        <is>
-          <t>8500</t>
-        </is>
-      </c>
-      <c r="M230" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>230</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>room_230_img1.webp</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr"/>
-      <c r="D231" t="inlineStr"/>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
-      <c r="G231" t="inlineStr">
-        <is>
-          <t>Smriti Nagar, Bhilai</t>
-        </is>
-      </c>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t>85459</t>
-        </is>
-      </c>
-      <c r="I231" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K231" t="inlineStr"/>
-      <c r="L231" t="inlineStr">
-        <is>
-          <t>3500</t>
-        </is>
-      </c>
-      <c r="M231" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>